<commit_message>
feat: add aotera listing
</commit_message>
<xml_diff>
--- a/ai-api-sites-table.xlsx
+++ b/ai-api-sites-table.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24000" windowHeight="12080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ai-api-sites-table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ai-api-sites-table" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14"/>
   <cols>
     <col width="7" customWidth="1" style="9" min="1" max="1"/>
@@ -2555,32 +2555,62 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="0" t="n">
         <v>52</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="0" t="inlineStr">
         <is>
           <t>New API</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>https://xxs.l.cd/sign-up?aff=RhO4</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>注册赠送;DeepSeek</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="0" t="inlineStr">
         <is>
           <t>注册送 50，只有 DeepSeek 可用</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="0" t="inlineStr">
         <is>
           <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>53</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>aotera</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://aotera.cc/sign-up?aff=gC8q</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>签到;GPT</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>邮箱注册 大额签到站，第一天送6，0.1倍率GPT，相当60刀。签到在个人资料</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>